<commit_message>
Serialize console paging and isolate catalog generations with regressions
</commit_message>
<xml_diff>
--- a/evidence/s03a/dom/console_finance.xlsx
+++ b/evidence/s03a/dom/console_finance.xlsx
@@ -87,7 +87,7 @@
     <t>snapshot_id</t>
   </si>
   <si>
-    <t>b969d05b5c8962609d2c12a6151c69ec</t>
+    <t>66d7c11e6288c6086aecc3243887460d</t>
   </si>
   <si>
     <t>integration_id</t>
@@ -105,7 +105,7 @@
     <t>as_of</t>
   </si>
   <si>
-    <t>2026-10-26</t>
+    <t>2026-10-27</t>
   </si>
   <si>
     <t>timezone</t>
@@ -117,7 +117,7 @@
     <t>query_hash</t>
   </si>
   <si>
-    <t>57ef45fcb414e8b9d4a75b7a83a6046a8c61216d35f8e1a0bca4dbafe9f33d25</t>
+    <t>0bda9cd8fc6ca0b7a3eddc8acec5a3c2ab1482f8a6ee902ea91722d4ce5b0a14</t>
   </si>
   <si>
     <t>source_watermark</t>
@@ -129,13 +129,13 @@
     <t>source_snapshot_ref</t>
   </si>
   <si>
-    <t>b5eeff2dc7f572db358680c4c5e9ac8e</t>
+    <t>9b13e0ed5c2c58f1c014c2b7a20e0571</t>
   </si>
   <si>
     <t>expires_at</t>
   </si>
   <si>
-    <t>2026-10-27T00:01:06+08:00</t>
+    <t>2026-10-27T00:27:09+08:00</t>
   </si>
   <si>
     <t>precision</t>

</xml_diff>

<commit_message>
Scope task refresh and cancel errors to their view and snapshot
</commit_message>
<xml_diff>
--- a/evidence/s03a/dom/console_finance.xlsx
+++ b/evidence/s03a/dom/console_finance.xlsx
@@ -87,7 +87,7 @@
     <t>snapshot_id</t>
   </si>
   <si>
-    <t>66d7c11e6288c6086aecc3243887460d</t>
+    <t>49f89caa6648f1ac69d14b40c2db7a68</t>
   </si>
   <si>
     <t>integration_id</t>
@@ -129,13 +129,13 @@
     <t>source_snapshot_ref</t>
   </si>
   <si>
-    <t>9b13e0ed5c2c58f1c014c2b7a20e0571</t>
+    <t>290619594861677eba095db77cb70730</t>
   </si>
   <si>
     <t>expires_at</t>
   </si>
   <si>
-    <t>2026-10-27T00:27:09+08:00</t>
+    <t>2026-10-27T00:32:53+08:00</t>
   </si>
   <si>
     <t>precision</t>

</xml_diff>

<commit_message>
Scope every task operation to its resource and stabilize catalog test latches
</commit_message>
<xml_diff>
--- a/evidence/s03a/dom/console_finance.xlsx
+++ b/evidence/s03a/dom/console_finance.xlsx
@@ -87,7 +87,7 @@
     <t>snapshot_id</t>
   </si>
   <si>
-    <t>49f89caa6648f1ac69d14b40c2db7a68</t>
+    <t>d38d8293bbf78202e66bc6825403134a</t>
   </si>
   <si>
     <t>integration_id</t>
@@ -129,13 +129,13 @@
     <t>source_snapshot_ref</t>
   </si>
   <si>
-    <t>290619594861677eba095db77cb70730</t>
+    <t>e1dec74badaf47839d45631de56b11a6</t>
   </si>
   <si>
     <t>expires_at</t>
   </si>
   <si>
-    <t>2026-10-27T00:32:53+08:00</t>
+    <t>2026-10-27T00:40:47+08:00</t>
   </si>
   <si>
     <t>precision</t>

</xml_diff>